<commit_message>
Documentação acadêmica do projeto iMX6 Rex
</commit_message>
<xml_diff>
--- a/PCB_Avancado/BoM/BOM_e_Cotacao.xlsx
+++ b/PCB_Avancado/BoM/BOM_e_Cotacao.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia_me" sheetId="1" r:id="R480ff65fa5f34ace"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM_Modulo" sheetId="2" r:id="R7d42aef3fccb44f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM_Base" sheetId="3" r:id="Rdd1dde73bb2941a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Itens_auxiliares" sheetId="4" r:id="Rc7a8c8d945b0479a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotacao" sheetId="5" r:id="Rdd21ecac5f1f443f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia_me" sheetId="1" r:id="R86f21fa28a214a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM_Modulo" sheetId="2" r:id="Rf13dee78f76c46fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM_Base" sheetId="3" r:id="Rf7af992569a94160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Itens_auxiliares" sheetId="4" r:id="Rf4402143d5614a17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cotacao" sheetId="5" r:id="Rc5809015fefc49ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -414,7 +414,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>PCB Avançado | BOM e cotação</x:v>
+        <x:v>PCB Avançado — Lista de materiais e cotação</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -442,7 +442,7 @@
     </x:row>
     <x:row r="3" ht="39" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Material</x:v>
+        <x:v>Projeto</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
         <x:v>iMX6 Rex — módulo e Development Baseboard</x:v>
@@ -547,7 +547,7 @@
         <x:v>Variante Prototype</x:v>
       </x:c>
       <x:c r="B9" s="6" t="str">
-        <x:v>29 registros de alteração no módulo e 76 na base. Revisar no Altium antes de montagem.</x:v>
+        <x:v>29 registros de configuração no módulo e 76 na placa base.</x:v>
       </x:c>
       <x:c r="C9" s="1"/>
       <x:c r="D9" s="1"/>
@@ -578,10 +578,10 @@
     </x:row>
     <x:row r="11" ht="39" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>Compra e montagem</x:v>
+        <x:v>Configuração</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>A seleção da variante e dos códigos da montadora deve ser validada antes de comprar.</x:v>
+        <x:v>BOM da configuração base. A variante Prototype possui registros próprios nos arquivos CSV.</x:v>
       </x:c>
       <x:c r="C11" s="1"/>
       <x:c r="D11" s="1"/>
@@ -598,7 +598,7 @@
         <x:v>Cotação</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>Valores em USD transcritos dos prints fornecidos; não é um pedido pago.</x:v>
+        <x:v>Orçamento JLCPCB em dólares americanos (USD), com fabricação e montagem da placa base.</x:v>
       </x:c>
       <x:c r="C12" s="1"/>
       <x:c r="D12" s="1"/>
@@ -615,7 +615,7 @@
         <x:v>Arquivos de apoio</x:v>
       </x:c>
       <x:c r="B13" s="6" t="str">
-        <x:v>Consulte os CSVs e READMEs na pasta BoM e os prints na pasta Cotacao.</x:v>
+        <x:v>BOMs em CSV na pasta BoM e orçamento detalhado na pasta Cotacao.</x:v>
       </x:c>
       <x:c r="C13" s="1"/>
       <x:c r="D13" s="1"/>
@@ -8191,7 +8191,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea703a6d31c846a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dd0497baf6b42be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13356,7 +13356,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4cf24d360564ceb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2d43779be5043d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13395,7 +13395,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1" t="str">
-        <x:v>Não somados à BOM principal; avaliar a necessidade de compra/montagem de cada item.</x:v>
+        <x:v>Elementos mecânicos, pontos de teste e referências complementares, separados da BOM principal.</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -17513,7 +17513,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91a16ce078f84cc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e361a9ebb004984"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17534,7 +17534,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>JLCPCB | cotação registrada nos prints</x:v>
+        <x:v>JLCPCB — Orçamento de fabricação e montagem</x:v>
       </x:c>
       <x:c r="B1" s="1"/>
       <x:c r="C1" s="1"/>
@@ -17549,7 +17549,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="1" t="str">
-        <x:v>USD • capturas com nomes datados de 12/10/2026 • pagamento não comprovado</x:v>
+        <x:v>Valores em dólares americanos (USD)</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -17599,7 +17599,7 @@
         <x:v>Valor do item (USD)</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
-        <x:v>Prazo exibido</x:v>
+        <x:v>Prazo de produção</x:v>
       </x:c>
       <x:c r="E5" s="10" t="str">
         <x:v>Configuração</x:v>
@@ -17695,7 +17695,7 @@
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
       <x:c r="A10" s="13" t="str">
-        <x:v>Soma dos itens, sem frete / tributos</x:v>
+        <x:v>Subtotal dos itens, sem frete e tributos</x:v>
       </x:c>
       <x:c r="B10" s="13"/>
       <x:c r="C10" s="25" t="n">
@@ -17726,7 +17726,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="1" t="str">
-        <x:v>Frete exibido para o módulo</x:v>
+        <x:v>Frete do módulo</x:v>
       </x:c>
       <x:c r="B12" s="1"/>
       <x:c r="C12" s="24" t="n">
@@ -17773,7 +17773,7 @@
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="7" t="str">
-        <x:v>Frete separado: não há cotação consolidada do envio das duas placas.</x:v>
+        <x:v>Subtotal de fabricação e montagem: frete e tributos separados.</x:v>
       </x:c>
       <x:c r="B15" s="1"/>
       <x:c r="C15" s="1"/>
@@ -17788,7 +17788,7 @@
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="7" t="str">
-        <x:v>Montagem da base: 2 unidades, dos dois lados. Compra de PCB: 5 unidades.</x:v>
+        <x:v>Placa base: fabricação de 5 PCBs e montagem de 2 unidades, nos dois lados.</x:v>
       </x:c>
       <x:c r="B16" s="1"/>
       <x:c r="C16" s="1"/>
@@ -17803,7 +17803,7 @@
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="7" t="str">
-        <x:v>Módulo HDI: a captura informa montagem PCBA indisponível.</x:v>
+        <x:v>Módulo HDI: serviço de montagem PCBA indisponível nesta cotação.</x:v>
       </x:c>
       <x:c r="B17" s="1"/>
       <x:c r="C17" s="1"/>
@@ -17817,9 +17817,7 @@
       <x:c r="K17" s="1"/>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
-      <x:c r="A18" s="7" t="str">
-        <x:v>Não há detalhamento suficiente para confirmar todos os componentes no preço de PCBA.</x:v>
-      </x:c>
+      <x:c r="A18" s="7"/>
       <x:c r="B18" s="1"/>
       <x:c r="C18" s="1"/>
       <x:c r="D18" s="1"/>
@@ -17832,9 +17830,7 @@
       <x:c r="K18" s="1"/>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
-      <x:c r="A19" s="7" t="str">
-        <x:v>O resumo US$ 0,00 do carrinho está com os itens desmarcados; não é o total dos itens.</x:v>
-      </x:c>
+      <x:c r="A19" s="7"/>
       <x:c r="B19" s="1"/>
       <x:c r="C19" s="1"/>
       <x:c r="D19" s="1"/>
@@ -17848,7 +17844,7 @@
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="7" t="str">
-        <x:v>Fontes: Cotacao/01_Cotacao_modulo_HDI.png e 02_Carrinho_PCB_e_montagem.png.</x:v>
+        <x:v>Referências: Cotacao/01_Cotacao_modulo_HDI.png e 02_Carrinho_PCB_e_montagem.png.</x:v>
       </x:c>
       <x:c r="B20" s="1"/>
       <x:c r="C20" s="1"/>
@@ -20984,7 +20980,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R850a39a98d0b403a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R827bb35c5e84482a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>